<commit_message>
actualizacion de requerimientos funcionales
</commit_message>
<xml_diff>
--- a/DSY1104 Evaluación Parcial 1 - Anexo 2 Planilla de Requerimientos.xlsx
+++ b/DSY1104 Evaluación Parcial 1 - Anexo 2 Planilla de Requerimientos.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chaij\OneDrive\Escritorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AO-Alumno\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77783C6A-B6BC-46AC-8925-B9E0AE807A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="4" r:id="rId1"/>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="176">
   <si>
     <t>[Nombre del Requerimiento]</t>
   </si>
@@ -327,12 +328,240 @@
   </si>
   <si>
     <t>Recuperación ante Caídas (feature B)</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir seleccionar una fecha y horario de entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir especificar la dirección de entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir indicar instrucciones especiales para la entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá mostrar un resumen de la sorpresa antes de confirmar la compra</t>
+  </si>
+  <si>
+    <t>El sistema deberá calcular automáticamente el precio total del pedido</t>
+  </si>
+  <si>
+    <t>R.29</t>
+  </si>
+  <si>
+    <t>R.30</t>
+  </si>
+  <si>
+    <t>R.31</t>
+  </si>
+  <si>
+    <t>R.32</t>
+  </si>
+  <si>
+    <t>R.33</t>
+  </si>
+  <si>
+    <t>R.34</t>
+  </si>
+  <si>
+    <t>R.35</t>
+  </si>
+  <si>
+    <t>R.36</t>
+  </si>
+  <si>
+    <t>R.37</t>
+  </si>
+  <si>
+    <t>R.38</t>
+  </si>
+  <si>
+    <t>R.39</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir crear campañas asociadas a fechas especiales</t>
+  </si>
+  <si>
+    <t>El administrador deberá poder configurar una fecha especial indicando nombre, descripción, imagen y período de vigencia</t>
+  </si>
+  <si>
+    <t>El administrador deberá poder asociar productos específicos a una fecha especial</t>
+  </si>
+  <si>
+    <t>El sistema deberá mostrar productos recomendados según la fecha especial seleccionada por el cliente</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir filtrar productos según la ocasión</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir realizar pedidos anticipados para fechas especiales</t>
+  </si>
+  <si>
+    <t>El sistema deberá notificar al usuario sobre próximas fechas especiales relevantes</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir al cliente solicitar la organización de un evento</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir seleccionar el tipo de evento</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir indicar la cantidad estimada de invitados</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir seleccionar la fecha del evento</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir indicar la ubicación del evento</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir seleccionar servicios adicionales</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir ingresar un presupuesto estimado</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir agregar comentarios o requerimientos especiales</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir solicitar una cotización personalizada</t>
+  </si>
+  <si>
+    <t>R.40</t>
+  </si>
+  <si>
+    <t>R.41</t>
+  </si>
+  <si>
+    <t>R.42</t>
+  </si>
+  <si>
+    <t>R.43</t>
+  </si>
+  <si>
+    <t>R.44</t>
+  </si>
+  <si>
+    <t>R.45</t>
+  </si>
+  <si>
+    <t>R.46</t>
+  </si>
+  <si>
+    <t>R.47</t>
+  </si>
+  <si>
+    <t>El administrador deberá poder revisar las solicitudes de cotización</t>
+  </si>
+  <si>
+    <t>El administrador deberá poder generar una cotización para el cliente</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir modificar los servicios incluidos en una cotización</t>
+  </si>
+  <si>
+    <t>El cliente deberá poder visualizar la cotización recibida</t>
+  </si>
+  <si>
+    <t>El cliente deberá poder aceptar o rechazar una cotización</t>
+  </si>
+  <si>
+    <t>El sistema deberá registrar el estado de cada cotización</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir al cliente revisar sus pedidos anteriores</t>
+  </si>
+  <si>
+    <t>El sistema deberá mostrar el estado actual del pedido</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir cancelar un pedido cuando cumpla las condiciones de cancelación establecidas</t>
+  </si>
+  <si>
+    <t>El administrador deberá poder actualizar el estado de un pedido</t>
+  </si>
+  <si>
+    <t>R.48</t>
+  </si>
+  <si>
+    <t>R.49</t>
+  </si>
+  <si>
+    <t>R.50</t>
+  </si>
+  <si>
+    <t>R.51</t>
+  </si>
+  <si>
+    <t>R.52</t>
+  </si>
+  <si>
+    <t>R.53</t>
+  </si>
+  <si>
+    <t>R.54</t>
+  </si>
+  <si>
+    <t>R.55</t>
+  </si>
+  <si>
+    <t>R.56</t>
+  </si>
+  <si>
+    <t>R.57</t>
+  </si>
+  <si>
+    <t>R.58</t>
+  </si>
+  <si>
+    <t>R.59</t>
+  </si>
+  <si>
+    <t>R.60</t>
+  </si>
+  <si>
+    <t>R.61</t>
+  </si>
+  <si>
+    <t>R.62</t>
+  </si>
+  <si>
+    <t>R.63</t>
+  </si>
+  <si>
+    <t>R.64</t>
+  </si>
+  <si>
+    <t>R.65</t>
+  </si>
+  <si>
+    <t>R.66</t>
+  </si>
+  <si>
+    <t>R.67</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir registrar información de entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir indicar una fecha y rango horario de entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá registrar el estado de la entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir al administrador asignar una entrega a un repartidor</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir registrar la confirmación de entrega</t>
+  </si>
+  <si>
+    <t>El sistema deberá permitir enviar al cliente una notificación cuando el pedido haya sido entregado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -387,7 +616,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -454,8 +683,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -493,11 +734,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="8"/>
+      </left>
+      <right style="thin">
+        <color theme="8"/>
+      </right>
+      <top style="thin">
+        <color theme="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0070C0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0070C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0070C0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF0070C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -542,32 +811,76 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -852,7 +1165,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -931,15 +1244,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" customWidth="1"/>
-    <col min="2" max="2" width="49.140625" customWidth="1"/>
+    <col min="2" max="2" width="56.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.5703125" customWidth="1"/>
     <col min="4" max="4" width="25.5703125" customWidth="1"/>
-    <col min="5" max="5" width="155.5703125" customWidth="1"/>
+    <col min="5" max="5" width="92.7109375" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1108,10 +1421,10 @@
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="23" t="s">
         <v>46</v>
       </c>
       <c r="C14" s="4"/>
@@ -1119,10 +1432,10 @@
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="23" t="s">
         <v>47</v>
       </c>
       <c r="C15" s="4"/>
@@ -1131,276 +1444,610 @@
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="F17" s="34" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="23" t="s">
+      <c r="B17" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+    </row>
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="F18" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="B18" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="41"/>
+    </row>
+    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="F19" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
+      <c r="B19" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+    </row>
+    <row r="20" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="31" t="s">
+      <c r="B20" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="41"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+    </row>
+    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="F21" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="23" t="s">
+      <c r="B21" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+    </row>
+    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="F22" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="31" t="s">
+      <c r="B22" s="45" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+    </row>
+    <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="F23" s="34" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="23" t="s">
+      <c r="B23" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+    </row>
+    <row r="24" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="F24" s="34" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="23" t="s">
+      <c r="B24" s="45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+    </row>
+    <row r="25" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="B25" s="29" t="s">
-        <v>83</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="F25" s="34" t="s">
-        <v>78</v>
-      </c>
+      <c r="B25" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="41"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="41"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="F26" s="35" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="23" t="s">
+      <c r="B26" s="44" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+    </row>
+    <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="B27" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="F27" s="35" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="B27" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="41"/>
+    </row>
+    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="33" t="s">
-        <v>92</v>
-      </c>
-      <c r="C28" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="D28" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E28" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="F28" s="35" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="23" t="s">
+      <c r="B28" s="45" t="s">
+        <v>122</v>
+      </c>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="41"/>
+    </row>
+    <row r="29" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="D29" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="F29" s="35" t="s">
-        <v>78</v>
-      </c>
+      <c r="B29" s="47" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="41"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="B30" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+    </row>
+    <row r="31" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="B31" s="47" t="s">
+        <v>125</v>
+      </c>
+      <c r="C31" s="41"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="41"/>
+      <c r="F31" s="41"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>126</v>
+      </c>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="B35" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
+    </row>
+    <row r="36" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="46" t="s">
+        <v>111</v>
+      </c>
+      <c r="B36" s="47" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+    </row>
+    <row r="37" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" s="47" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="41"/>
+    </row>
+    <row r="38" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="50" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" s="51" t="s">
+        <v>140</v>
+      </c>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+    </row>
+    <row r="39" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="B39" s="51" t="s">
+        <v>141</v>
+      </c>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+    </row>
+    <row r="40" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="50" t="s">
+        <v>115</v>
+      </c>
+      <c r="B40" s="51" t="s">
+        <v>142</v>
+      </c>
+      <c r="C40" s="41"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="41"/>
+      <c r="F40" s="41"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C42" s="41"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="41"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="B43" s="51" t="s">
+        <v>145</v>
+      </c>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+    </row>
+    <row r="44" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="52" t="s">
+        <v>135</v>
+      </c>
+      <c r="B44" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="C44" s="41"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="52" t="s">
+        <v>136</v>
+      </c>
+      <c r="B45" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="41"/>
+    </row>
+    <row r="46" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="52" t="s">
+        <v>137</v>
+      </c>
+      <c r="B46" s="53" t="s">
+        <v>148</v>
+      </c>
+      <c r="C46" s="41"/>
+      <c r="D46" s="41"/>
+      <c r="E46" s="41"/>
+      <c r="F46" s="41"/>
+    </row>
+    <row r="47" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="52" t="s">
+        <v>138</v>
+      </c>
+      <c r="B47" s="53" t="s">
+        <v>149</v>
+      </c>
+      <c r="C47" s="41"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="41"/>
+      <c r="F47" s="41"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="54" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" s="55" t="s">
+        <v>170</v>
+      </c>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+    </row>
+    <row r="49" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="54" t="s">
+        <v>150</v>
+      </c>
+      <c r="B49" s="55" t="s">
+        <v>171</v>
+      </c>
+      <c r="C49" s="41"/>
+      <c r="D49" s="41"/>
+      <c r="E49" s="41"/>
+      <c r="F49" s="41"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="54" t="s">
+        <v>151</v>
+      </c>
+      <c r="B50" s="55" t="s">
+        <v>172</v>
+      </c>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
+      <c r="F50" s="41"/>
+    </row>
+    <row r="51" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="54" t="s">
+        <v>152</v>
+      </c>
+      <c r="B51" s="55" t="s">
+        <v>173</v>
+      </c>
+      <c r="C51" s="41"/>
+      <c r="D51" s="41"/>
+      <c r="E51" s="41"/>
+      <c r="F51" s="41"/>
+    </row>
+    <row r="52" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="54" t="s">
+        <v>153</v>
+      </c>
+      <c r="B52" s="55" t="s">
+        <v>174</v>
+      </c>
+      <c r="C52" s="41"/>
+      <c r="D52" s="41"/>
+      <c r="E52" s="41"/>
+      <c r="F52" s="41"/>
+    </row>
+    <row r="53" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="54" t="s">
+        <v>154</v>
+      </c>
+      <c r="B53" s="55" t="s">
+        <v>175</v>
+      </c>
+      <c r="C53" s="41"/>
+      <c r="D53" s="41"/>
+      <c r="E53" s="41"/>
+      <c r="F53" s="41"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="48" t="s">
+        <v>155</v>
+      </c>
+      <c r="B54" s="49"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="41"/>
+      <c r="F54" s="41"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="48" t="s">
+        <v>156</v>
+      </c>
+      <c r="B55" s="49"/>
+      <c r="C55" s="41"/>
+      <c r="D55" s="41"/>
+      <c r="E55" s="41"/>
+      <c r="F55" s="41"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="48" t="s">
+        <v>157</v>
+      </c>
+      <c r="B56" s="49"/>
+      <c r="C56" s="41"/>
+      <c r="D56" s="41"/>
+      <c r="E56" s="41"/>
+      <c r="F56" s="41"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="48" t="s">
+        <v>158</v>
+      </c>
+      <c r="B57" s="49"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="48" t="s">
+        <v>159</v>
+      </c>
+      <c r="B58" s="49"/>
+      <c r="C58" s="41"/>
+      <c r="D58" s="41"/>
+      <c r="E58" s="41"/>
+      <c r="F58" s="41"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="48" t="s">
+        <v>160</v>
+      </c>
+      <c r="B59" s="49"/>
+      <c r="C59" s="41"/>
+      <c r="D59" s="41"/>
+      <c r="E59" s="41"/>
+      <c r="F59" s="41"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="48" t="s">
+        <v>161</v>
+      </c>
+      <c r="B60" s="49"/>
+      <c r="C60" s="41"/>
+      <c r="D60" s="41"/>
+      <c r="E60" s="41"/>
+      <c r="F60" s="41"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="B61" s="49"/>
+      <c r="C61" s="41"/>
+      <c r="D61" s="41"/>
+      <c r="E61" s="41"/>
+      <c r="F61" s="41"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="B62" s="49"/>
+      <c r="C62" s="41"/>
+      <c r="D62" s="41"/>
+      <c r="E62" s="41"/>
+      <c r="F62" s="41"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="48" t="s">
+        <v>164</v>
+      </c>
+      <c r="B63" s="49"/>
+      <c r="C63" s="41"/>
+      <c r="D63" s="41"/>
+      <c r="E63" s="41"/>
+      <c r="F63" s="41"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="B64" s="49"/>
+      <c r="C64" s="41"/>
+      <c r="D64" s="41"/>
+      <c r="E64" s="41"/>
+      <c r="F64" s="41"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="48" t="s">
+        <v>166</v>
+      </c>
+      <c r="B65" s="49"/>
+      <c r="C65" s="41"/>
+      <c r="D65" s="41"/>
+      <c r="E65" s="41"/>
+      <c r="F65" s="41"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="48" t="s">
+        <v>167</v>
+      </c>
+      <c r="B66" s="49"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="48" t="s">
+        <v>168</v>
+      </c>
+      <c r="B67" s="49"/>
+      <c r="C67" s="41"/>
+      <c r="D67" s="41"/>
+      <c r="E67" s="41"/>
+      <c r="F67" s="41"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="48" t="s">
+        <v>169</v>
+      </c>
+      <c r="B68" s="49"/>
+      <c r="C68" s="41"/>
+      <c r="D68" s="41"/>
+      <c r="E68" s="41"/>
+      <c r="F68" s="41"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -1410,7 +2057,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1442,137 +2089,267 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-    </row>
-    <row r="3" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-    </row>
-    <row r="6" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-    </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" s="31" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -1582,7 +2359,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>17</v>
       </c>
@@ -1598,6 +2375,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e1e7bc46-bed0-459f-9452-a76b1c5b695e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005395107FFD641345A10C8A5ACACB9D20" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ce7786e0ad11988b1588e06b80e33958">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e1e7bc46-bed0-459f-9452-a76b1c5b695e" xmlns:ns3="bb8cf7e1-610f-40a0-8f00-126b9d139fde" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="99ef8fa6ee73c11c731191fdf3d87e67" ns2:_="" ns3:_="">
     <xsd:import namespace="e1e7bc46-bed0-459f-9452-a76b1c5b695e"/>
@@ -1808,26 +2604,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e1e7bc46-bed0-459f-9452-a76b1c5b695e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{370A914A-1DD7-4F78-8671-F61C286C2CC1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14168F1D-C031-4047-A789-A93363341739}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e1e7bc46-bed0-459f-9452-a76b1c5b695e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F4FA5F9-E1BF-40AC-BEF4-FE15B10C9F42}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1844,22 +2639,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14168F1D-C031-4047-A789-A93363341739}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e1e7bc46-bed0-459f-9452-a76b1c5b695e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{370A914A-1DD7-4F78-8671-F61C286C2CC1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>